<commit_message>
Task matrix: P1-16, P1-21, P1-26 done (confirmed in Studio)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bjoj9kNHaBJ7Zd78F1MCBY
</commit_message>
<xml_diff>
--- a/testing/Central_Deposit_-_Task_Matrix_v3_status-23-09.xlsx
+++ b/testing/Central_Deposit_-_Task_Matrix_v3_status-23-09.xlsx
@@ -1948,9 +1948,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="E19" s="44" t="inlineStr">
-        <is>
-          <t>Ready for Dev</t>
+      <c r="E19" s="54" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F19" s="45" t="n"/>
@@ -1968,12 +1968,12 @@
       </c>
       <c r="K19" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Done in Studio (confirmed by Alexander, 23/09): Case 2 label corrected.</t>
         </is>
       </c>
       <c r="L19" s="42" t="inlineStr">
         <is>
-          <t>Not done: the Contract case list still reads "Case 2 - specific service contract" (Case 1 reads "framework / direct service contract"). Confirm the wording; one-line change in CL_Case.Items.</t>
+          <t>Nothing in the app. Not in the v44 file, so keep this change when the next version is merged.</t>
         </is>
       </c>
     </row>
@@ -2186,9 +2186,9 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="E24" s="52" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="E24" s="54" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F24" s="45" t="n"/>
@@ -2202,12 +2202,12 @@
       <c r="J24" s="53" t="n"/>
       <c r="K24" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Done in Studio (confirmed by Alexander, 23/09): Request Management opens with sections expanded.</t>
         </is>
       </c>
       <c r="L24" s="42" t="inlineStr">
         <is>
-          <t>Not done: the filter sections still open collapsed (locShowFilters starts false).</t>
+          <t>Nothing in the app. Not in the v44 file, so keep this change when the next version is merged.</t>
         </is>
       </c>
     </row>
@@ -2416,9 +2416,9 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="E29" s="52" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="E29" s="54" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F29" s="45" t="n"/>
@@ -2432,12 +2432,12 @@
       <c r="J29" s="53" t="n"/>
       <c r="K29" s="42" t="inlineStr">
         <is>
-          <t>v12 restyled it, but the current app has "+ Media" orange (RGBA 180, 95, 6) while Submit is blue (RGBA 56, 96, 178).</t>
+          <t>Done in Studio (confirmed by Alexander, 23/09): "+ Media" button styled like Submit.</t>
         </is>
       </c>
       <c r="L29" s="42" t="inlineStr">
         <is>
-          <t>Not done in the current app: set RS_BtnDraftSave_1 colours to match Submit.</t>
+          <t>Nothing in the app. Not in the v44 file, so keep this change when the next version is merged.</t>
         </is>
       </c>
     </row>

</xml_diff>